<commit_message>
Update downloadable case study workbook with latest edits
Confirmed the 3 sheets featured in full on the site (Week 1, Week 7,
Executive Review) are unchanged -- no page copy needed updating.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/case-study/Cypress-Manufacturing-Payroll-Case-Study.xlsx
+++ b/assets/case-study/Cypress-Manufacturing-Payroll-Case-Study.xlsx
@@ -3,10 +3,10 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{477FDEDE-B894-5743-A9F4-0D923AEC60FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{958E5648-DFE6-DC4A-A98F-095A561D46F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="16060" xr2:uid="{C4273654-4867-1941-B027-2D844191C07C}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="16060" activeTab="7" xr2:uid="{C4273654-4867-1941-B027-2D844191C07C}"/>
   </bookViews>
   <sheets>
     <sheet name="Case Study Structure" sheetId="2" r:id="rId1"/>
@@ -2485,32 +2485,23 @@
     <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="27" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="6" fontId="10" fillId="5" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="25" fillId="4" borderId="0" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="17" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -2530,11 +2521,20 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -2935,6 +2935,51 @@
       </font>
     </dxf>
     <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="12" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="21" formatCode="d\-mmm"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="164" formatCode="0.0%"/>
     </dxf>
     <dxf>
@@ -3211,51 +3256,6 @@
         <bottom/>
       </border>
     </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="12" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="21" formatCode="d\-mmm"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -3270,7 +3270,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{383E5A6A-9EA9-DC47-B482-CE4D1C46D702}" name="Table1" displayName="Table1" ref="A5:D6" totalsRowShown="0" headerRowDxfId="70" headerRowBorderDxfId="69" tableBorderDxfId="68" totalsRowBorderDxfId="67">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{383E5A6A-9EA9-DC47-B482-CE4D1C46D702}" name="Table1" displayName="Table1" ref="A5:D6" totalsRowShown="0" headerRowDxfId="75" headerRowBorderDxfId="74" tableBorderDxfId="73" totalsRowBorderDxfId="72">
   <autoFilter ref="A5:D6" xr:uid="{383E5A6A-9EA9-DC47-B482-CE4D1C46D702}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -3278,10 +3278,10 @@
     <filterColumn colId="3" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{AEDF3CE8-2DEB-EE45-8C53-1F85628633A7}" name="Industry" dataDxfId="66"/>
-    <tableColumn id="2" xr3:uid="{0B994CEB-94AD-4140-97F8-CDD33306A830}" name="Software" dataDxfId="65"/>
-    <tableColumn id="3" xr3:uid="{65967071-3AC9-3942-AA02-B3F2B5DB301B}" name="Headquarters" dataDxfId="64"/>
-    <tableColumn id="4" xr3:uid="{1BD4C854-3956-9E49-957F-40F4FCA0FAD5}" name="Pay Frequency" dataDxfId="63"/>
+    <tableColumn id="1" xr3:uid="{AEDF3CE8-2DEB-EE45-8C53-1F85628633A7}" name="Industry" dataDxfId="71"/>
+    <tableColumn id="2" xr3:uid="{0B994CEB-94AD-4140-97F8-CDD33306A830}" name="Software" dataDxfId="70"/>
+    <tableColumn id="3" xr3:uid="{65967071-3AC9-3942-AA02-B3F2B5DB301B}" name="Headquarters" dataDxfId="69"/>
+    <tableColumn id="4" xr3:uid="{1BD4C854-3956-9E49-957F-40F4FCA0FAD5}" name="Pay Frequency" dataDxfId="68"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium20" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3394,7 +3394,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{6FE775DD-B461-4347-8D3F-819C8C31609A}" name="Table2" displayName="Table2" ref="A14:J24" totalsRowShown="0" headerRowDxfId="62">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{6FE775DD-B461-4347-8D3F-819C8C31609A}" name="Table2" displayName="Table2" ref="A14:J24" totalsRowShown="0" headerRowDxfId="67">
   <autoFilter ref="A14:J24" xr:uid="{6FE775DD-B461-4347-8D3F-819C8C31609A}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -3416,15 +3416,15 @@
     <tableColumn id="6" xr3:uid="{224D6D44-F303-774C-A528-92B3AA22879B}" name="Pay Type"/>
     <tableColumn id="7" xr3:uid="{868140BC-A833-124B-A94F-8B5A38DEF6A5}" name="Regular Hours"/>
     <tableColumn id="8" xr3:uid="{E671470B-0A1C-874B-A4AA-533A39A3CFA8}" name="OT Hours"/>
-    <tableColumn id="9" xr3:uid="{950491E5-BEFA-CA4D-A832-6FE31057E0B7}" name="Hourly Rate" dataDxfId="61"/>
-    <tableColumn id="10" xr3:uid="{680896A4-4C9A-0F48-AACB-EA763B9AB3A2}" name="Gross Pay" dataDxfId="60"/>
+    <tableColumn id="9" xr3:uid="{950491E5-BEFA-CA4D-A832-6FE31057E0B7}" name="Hourly Rate" dataDxfId="66"/>
+    <tableColumn id="10" xr3:uid="{680896A4-4C9A-0F48-AACB-EA763B9AB3A2}" name="Gross Pay" dataDxfId="65"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium6" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{2A7F74B7-2140-0943-A44D-A7F630110CEF}" name="Table3" displayName="Table3" ref="A44:E54" totalsRowShown="0" headerRowDxfId="59" dataDxfId="57" headerRowBorderDxfId="58" tableBorderDxfId="56">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{2A7F74B7-2140-0943-A44D-A7F630110CEF}" name="Table3" displayName="Table3" ref="A44:E54" totalsRowShown="0" headerRowDxfId="64" dataDxfId="62" headerRowBorderDxfId="63" tableBorderDxfId="61">
   <autoFilter ref="A44:E54" xr:uid="{2A7F74B7-2140-0943-A44D-A7F630110CEF}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -3434,9 +3434,9 @@
   </autoFilter>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{F501A1CD-2634-1E45-B325-ED46A02A8C59}" name="Employee"/>
-    <tableColumn id="2" xr3:uid="{094C7B36-23E9-2D46-A3B4-89252F172225}" name="Observation" dataDxfId="55"/>
-    <tableColumn id="3" xr3:uid="{D96B0134-ADDF-A34C-A43B-70661D422E93}" name="Why It Matters" dataDxfId="54"/>
-    <tableColumn id="4" xr3:uid="{A8571B47-41AC-0A43-A0AF-72A79C41C66E}" name="Recommended Next Step" dataDxfId="53"/>
+    <tableColumn id="2" xr3:uid="{094C7B36-23E9-2D46-A3B4-89252F172225}" name="Observation" dataDxfId="60"/>
+    <tableColumn id="3" xr3:uid="{D96B0134-ADDF-A34C-A43B-70661D422E93}" name="Why It Matters" dataDxfId="59"/>
+    <tableColumn id="4" xr3:uid="{A8571B47-41AC-0A43-A0AF-72A79C41C66E}" name="Recommended Next Step" dataDxfId="58"/>
     <tableColumn id="5" xr3:uid="{2592205F-EC3A-0546-A69E-71189210BB12}" name="Priority"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium6" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -3444,7 +3444,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{351AEDD7-0B28-4149-813B-66FA9F159C6C}" name="Table4" displayName="Table4" ref="A16:F23" totalsRowShown="0" headerRowDxfId="52">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{351AEDD7-0B28-4149-813B-66FA9F159C6C}" name="Table4" displayName="Table4" ref="A16:F23" totalsRowShown="0" headerRowDxfId="57">
   <autoFilter ref="A16:F23" xr:uid="{351AEDD7-0B28-4149-813B-66FA9F159C6C}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -3458,15 +3458,15 @@
     <tableColumn id="2" xr3:uid="{028E131D-1589-154E-A6BC-D933B354CFCA}" name="Previous OT Hours"/>
     <tableColumn id="3" xr3:uid="{B62BADED-F710-404F-82FD-857F0A99A4C2}" name="Current OT Hours"/>
     <tableColumn id="4" xr3:uid="{AF395F61-6C52-6C48-B882-4C60B174C066}" name="Change"/>
-    <tableColumn id="5" xr3:uid="{1A5D0D21-0C3C-5846-8142-100D11DE10BC}" name="Previous OT Cost" dataDxfId="51"/>
-    <tableColumn id="6" xr3:uid="{445B8E35-D644-904D-A104-13802A5197F3}" name="Current OT Cost" dataDxfId="50"/>
+    <tableColumn id="5" xr3:uid="{1A5D0D21-0C3C-5846-8142-100D11DE10BC}" name="Previous OT Cost" dataDxfId="56"/>
+    <tableColumn id="6" xr3:uid="{445B8E35-D644-904D-A104-13802A5197F3}" name="Current OT Cost" dataDxfId="55"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium6" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{0EF008CC-394B-6344-AF94-A7DCA1F43A7B}" name="Table5" displayName="Table5" ref="A63:K71" totalsRowShown="0" headerRowDxfId="49">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{0EF008CC-394B-6344-AF94-A7DCA1F43A7B}" name="Table5" displayName="Table5" ref="A63:K71" totalsRowShown="0" headerRowDxfId="54">
   <autoFilter ref="A63:K71" xr:uid="{0EF008CC-394B-6344-AF94-A7DCA1F43A7B}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -3485,12 +3485,12 @@
     <tableColumn id="2" xr3:uid="{D1DFEE06-891B-0A43-AB23-F4B8B17E8764}" name="Previous OT Hours"/>
     <tableColumn id="3" xr3:uid="{E07B0018-BC29-DD48-93E8-A71A47034A50}" name="Current OT Hours"/>
     <tableColumn id="4" xr3:uid="{D3727CA9-7D49-1648-8211-1BD086564169}" name="OT Variance"/>
-    <tableColumn id="5" xr3:uid="{0F4DF983-C252-1E4E-B5A2-FF2561B38668}" name="% Change/Increase (Hours)" dataDxfId="48" dataCellStyle="Percent"/>
-    <tableColumn id="6" xr3:uid="{37F4AE63-1CD6-EF4C-9115-9FD3C30C84F3}" name="Previous OT Cost" dataDxfId="47"/>
-    <tableColumn id="7" xr3:uid="{D1F9C495-D850-CB48-916B-84D9499A9448}" name="Current OT Cost" dataDxfId="46"/>
-    <tableColumn id="8" xr3:uid="{03A9D69E-29BB-624F-84D0-A5DFE8B0A3A3}" name="OT Cost Variance" dataDxfId="45"/>
-    <tableColumn id="9" xr3:uid="{4B69023F-FD00-D140-AFDE-B6E3A801B121}" name="% Change/Increase (Cost)" dataDxfId="44" dataCellStyle="Percent"/>
-    <tableColumn id="10" xr3:uid="{0C1A6056-F07A-8340-AC97-8AB86E910DC5}" name="Contribution to Total Increase" dataDxfId="43"/>
+    <tableColumn id="5" xr3:uid="{0F4DF983-C252-1E4E-B5A2-FF2561B38668}" name="% Change/Increase (Hours)" dataDxfId="53" dataCellStyle="Percent"/>
+    <tableColumn id="6" xr3:uid="{37F4AE63-1CD6-EF4C-9115-9FD3C30C84F3}" name="Previous OT Cost" dataDxfId="52"/>
+    <tableColumn id="7" xr3:uid="{D1F9C495-D850-CB48-916B-84D9499A9448}" name="Current OT Cost" dataDxfId="51"/>
+    <tableColumn id="8" xr3:uid="{03A9D69E-29BB-624F-84D0-A5DFE8B0A3A3}" name="OT Cost Variance" dataDxfId="50"/>
+    <tableColumn id="9" xr3:uid="{4B69023F-FD00-D140-AFDE-B6E3A801B121}" name="% Change/Increase (Cost)" dataDxfId="49" dataCellStyle="Percent"/>
+    <tableColumn id="10" xr3:uid="{0C1A6056-F07A-8340-AC97-8AB86E910DC5}" name="Contribution to Total Increase" dataDxfId="48"/>
     <tableColumn id="11" xr3:uid="{9A38B402-FD83-5249-80A6-81FFB1FDEDE2}" name="Notes"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium6" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -3498,7 +3498,7 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{94DD0E59-552A-004A-AE6C-3461962A0666}" name="Table6" displayName="Table6" ref="A18:G28" totalsRowShown="0" headerRowDxfId="75">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{94DD0E59-552A-004A-AE6C-3461962A0666}" name="Table6" displayName="Table6" ref="A18:G28" totalsRowShown="0" headerRowDxfId="47">
   <autoFilter ref="A18:G28" xr:uid="{94DD0E59-552A-004A-AE6C-3461962A0666}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -3511,7 +3511,7 @@
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{6E7464B2-2E9D-BC4B-BACE-FCCA89663E10}" name="Employee"/>
     <tableColumn id="2" xr3:uid="{6E0AF0A4-5FBE-FA40-96D1-32AE0AAB9F99}" name="Department"/>
-    <tableColumn id="3" xr3:uid="{6BAB4C3B-FB41-604B-8388-79605B985199}" name="Date" dataDxfId="74"/>
+    <tableColumn id="3" xr3:uid="{6BAB4C3B-FB41-604B-8388-79605B985199}" name="Date" dataDxfId="46"/>
     <tableColumn id="4" xr3:uid="{D0A68926-DC3B-074D-9592-84E6C512199E}" name="Shift Hours"/>
     <tableColumn id="5" xr3:uid="{76E90D76-F085-4F48-AE39-8EE88D5C33DA}" name="Meal Break"/>
     <tableColumn id="6" xr3:uid="{FA9160F9-C4F5-2243-BE46-63983AABFEA4}" name="Premium Paid"/>
@@ -3522,7 +3522,7 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{40F5E122-6DFE-6045-8A75-1C80ACE768C1}" name="Table7" displayName="Table7" ref="A63:F74" totalsRowShown="0" headerRowDxfId="73">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{40F5E122-6DFE-6045-8A75-1C80ACE768C1}" name="Table7" displayName="Table7" ref="A63:F74" totalsRowShown="0" headerRowDxfId="45">
   <autoFilter ref="A63:F74" xr:uid="{40F5E122-6DFE-6045-8A75-1C80ACE768C1}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -3536,8 +3536,8 @@
     <tableColumn id="2" xr3:uid="{8379B859-ADC9-0A45-9488-7A8D98D4FE19}" name="Exception"/>
     <tableColumn id="3" xr3:uid="{B5FFCA04-440B-5044-A809-AD21B4512853}" name="Evidence"/>
     <tableColumn id="4" xr3:uid="{D20F569C-B6FC-774E-8651-D3A95806B131}" name="Does It Require Review?"/>
-    <tableColumn id="5" xr3:uid="{388A88A7-6C48-B64D-A56E-A50F28A25F64}" name="Potential Premium" dataDxfId="72"/>
-    <tableColumn id="6" xr3:uid="{30ACDD88-9666-3F40-BD0E-7CF6A6A94BFE}" name="Questions" dataDxfId="71"/>
+    <tableColumn id="5" xr3:uid="{388A88A7-6C48-B64D-A56E-A50F28A25F64}" name="Potential Premium" dataDxfId="44"/>
+    <tableColumn id="6" xr3:uid="{30ACDD88-9666-3F40-BD0E-7CF6A6A94BFE}" name="Questions" dataDxfId="43"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium6" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3938,10 +3938,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="32" x14ac:dyDescent="0.4">
-      <c r="A1" s="82" t="s">
+      <c r="A1" s="77" t="s">
         <v>42</v>
       </c>
-      <c r="B1" s="82"/>
+      <c r="B1" s="77"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="78" t="s">
@@ -3988,20 +3988,20 @@
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A8" s="79" t="s">
+      <c r="A8" s="75" t="s">
         <v>483</v>
       </c>
-      <c r="B8" s="79"/>
-      <c r="C8" s="79"/>
-      <c r="D8" s="79"/>
+      <c r="B8" s="75"/>
+      <c r="C8" s="75"/>
+      <c r="D8" s="75"/>
     </row>
     <row r="9" spans="1:6" ht="27" x14ac:dyDescent="0.2">
-      <c r="A9" s="81" t="s">
+      <c r="A9" s="79" t="s">
         <v>529</v>
       </c>
-      <c r="B9" s="81"/>
-      <c r="C9" s="81"/>
-      <c r="D9" s="81"/>
+      <c r="B9" s="79"/>
+      <c r="C9" s="79"/>
+      <c r="D9" s="79"/>
     </row>
     <row r="10" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="78" t="s">
@@ -4015,20 +4015,20 @@
       <c r="A11" s="17"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A12" s="79" t="s">
+      <c r="A12" s="75" t="s">
         <v>484</v>
       </c>
-      <c r="B12" s="79"/>
-      <c r="C12" s="79"/>
-      <c r="D12" s="79"/>
+      <c r="B12" s="75"/>
+      <c r="C12" s="75"/>
+      <c r="D12" s="75"/>
     </row>
     <row r="13" spans="1:6" ht="27" x14ac:dyDescent="0.2">
-      <c r="A13" s="81" t="s">
+      <c r="A13" s="79" t="s">
         <v>530</v>
       </c>
-      <c r="B13" s="81"/>
-      <c r="C13" s="81"/>
-      <c r="D13" s="81"/>
+      <c r="B13" s="79"/>
+      <c r="C13" s="79"/>
+      <c r="D13" s="79"/>
     </row>
     <row r="14" spans="1:6" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="78" t="s">
@@ -4042,130 +4042,130 @@
       <c r="A15" s="17"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A16" s="79" t="s">
+      <c r="A16" s="75" t="s">
         <v>485</v>
       </c>
-      <c r="B16" s="79"/>
-      <c r="C16" s="79"/>
-      <c r="D16" s="79"/>
+      <c r="B16" s="75"/>
+      <c r="C16" s="75"/>
+      <c r="D16" s="75"/>
     </row>
     <row r="17" spans="1:4" ht="27" x14ac:dyDescent="0.2">
-      <c r="A17" s="81" t="s">
+      <c r="A17" s="79" t="s">
         <v>531</v>
       </c>
-      <c r="B17" s="81"/>
-      <c r="C17" s="81"/>
-      <c r="D17" s="81"/>
+      <c r="B17" s="79"/>
+      <c r="C17" s="79"/>
+      <c r="D17" s="79"/>
     </row>
     <row r="18" spans="1:4" ht="35" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="80" t="s">
+      <c r="A18" s="76" t="s">
         <v>473</v>
       </c>
-      <c r="B18" s="80"/>
-      <c r="C18" s="80"/>
-      <c r="D18" s="80"/>
+      <c r="B18" s="76"/>
+      <c r="C18" s="76"/>
+      <c r="D18" s="76"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" s="1"/>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A20" s="79" t="s">
+      <c r="A20" s="75" t="s">
         <v>486</v>
       </c>
-      <c r="B20" s="79"/>
-      <c r="C20" s="79"/>
-      <c r="D20" s="79"/>
+      <c r="B20" s="75"/>
+      <c r="C20" s="75"/>
+      <c r="D20" s="75"/>
     </row>
     <row r="21" spans="1:4" ht="27" x14ac:dyDescent="0.2">
-      <c r="A21" s="81" t="s">
+      <c r="A21" s="79" t="s">
         <v>532</v>
       </c>
-      <c r="B21" s="81"/>
-      <c r="C21" s="81"/>
-      <c r="D21" s="81"/>
+      <c r="B21" s="79"/>
+      <c r="C21" s="79"/>
+      <c r="D21" s="79"/>
     </row>
     <row r="22" spans="1:4" ht="34" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="80" t="s">
+      <c r="A22" s="76" t="s">
         <v>474</v>
       </c>
-      <c r="B22" s="80"/>
-      <c r="C22" s="80"/>
-      <c r="D22" s="80"/>
+      <c r="B22" s="76"/>
+      <c r="C22" s="76"/>
+      <c r="D22" s="76"/>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A24" s="79" t="s">
+      <c r="A24" s="75" t="s">
         <v>487</v>
       </c>
-      <c r="B24" s="79"/>
-      <c r="C24" s="79"/>
-      <c r="D24" s="79"/>
+      <c r="B24" s="75"/>
+      <c r="C24" s="75"/>
+      <c r="D24" s="75"/>
     </row>
     <row r="25" spans="1:4" ht="27" x14ac:dyDescent="0.2">
-      <c r="A25" s="81" t="s">
+      <c r="A25" s="79" t="s">
         <v>533</v>
       </c>
-      <c r="B25" s="81"/>
-      <c r="C25" s="81"/>
-      <c r="D25" s="81"/>
+      <c r="B25" s="79"/>
+      <c r="C25" s="79"/>
+      <c r="D25" s="79"/>
     </row>
     <row r="26" spans="1:4" ht="35" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="80" t="s">
+      <c r="A26" s="76" t="s">
         <v>475</v>
       </c>
-      <c r="B26" s="80"/>
-      <c r="C26" s="80"/>
-      <c r="D26" s="80"/>
+      <c r="B26" s="76"/>
+      <c r="C26" s="76"/>
+      <c r="D26" s="76"/>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A27" s="1"/>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A28" s="79" t="s">
+      <c r="A28" s="75" t="s">
         <v>488</v>
       </c>
-      <c r="B28" s="79"/>
-      <c r="C28" s="79"/>
-      <c r="D28" s="79"/>
+      <c r="B28" s="75"/>
+      <c r="C28" s="75"/>
+      <c r="D28" s="75"/>
     </row>
     <row r="29" spans="1:4" ht="27" x14ac:dyDescent="0.2">
-      <c r="A29" s="81" t="s">
+      <c r="A29" s="79" t="s">
         <v>534</v>
       </c>
-      <c r="B29" s="81"/>
-      <c r="C29" s="81"/>
-      <c r="D29" s="81"/>
+      <c r="B29" s="79"/>
+      <c r="C29" s="79"/>
+      <c r="D29" s="79"/>
     </row>
     <row r="30" spans="1:4" ht="38" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="80" t="s">
+      <c r="A30" s="76" t="s">
         <v>493</v>
       </c>
-      <c r="B30" s="80"/>
-      <c r="C30" s="80"/>
-      <c r="D30" s="80"/>
+      <c r="B30" s="76"/>
+      <c r="C30" s="76"/>
+      <c r="D30" s="76"/>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A32" s="79" t="s">
+      <c r="A32" s="75" t="s">
         <v>489</v>
       </c>
-      <c r="B32" s="79"/>
-      <c r="C32" s="79"/>
-      <c r="D32" s="79"/>
+      <c r="B32" s="75"/>
+      <c r="C32" s="75"/>
+      <c r="D32" s="75"/>
     </row>
     <row r="33" spans="1:5" ht="27" x14ac:dyDescent="0.2">
-      <c r="A33" s="81" t="s">
+      <c r="A33" s="79" t="s">
         <v>373</v>
       </c>
-      <c r="B33" s="81"/>
-      <c r="C33" s="81"/>
-      <c r="D33" s="81"/>
+      <c r="B33" s="79"/>
+      <c r="C33" s="79"/>
+      <c r="D33" s="79"/>
     </row>
     <row r="34" spans="1:5" ht="37" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="80" t="s">
+      <c r="A34" s="76" t="s">
         <v>494</v>
       </c>
-      <c r="B34" s="80"/>
-      <c r="C34" s="80"/>
-      <c r="D34" s="80"/>
+      <c r="B34" s="76"/>
+      <c r="C34" s="76"/>
+      <c r="D34" s="76"/>
     </row>
     <row r="35" spans="1:5" ht="19" x14ac:dyDescent="0.25">
       <c r="C35" s="31"/>
@@ -4183,14 +4183,8 @@
       <c r="E37" s="1"/>
     </row>
   </sheetData>
+  <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="23">
-    <mergeCell ref="A20:D20"/>
-    <mergeCell ref="A22:D22"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A8:D8"/>
-    <mergeCell ref="A10:D10"/>
-    <mergeCell ref="A12:D12"/>
-    <mergeCell ref="A14:D14"/>
     <mergeCell ref="A32:D32"/>
     <mergeCell ref="A34:D34"/>
     <mergeCell ref="A2:C2"/>
@@ -4207,6 +4201,13 @@
     <mergeCell ref="A28:D28"/>
     <mergeCell ref="A30:D30"/>
     <mergeCell ref="A18:D18"/>
+    <mergeCell ref="A20:D20"/>
+    <mergeCell ref="A22:D22"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A8:D8"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="A12:D12"/>
+    <mergeCell ref="A14:D14"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A8:D8" location="'Monday Morning Payroll Week 1'!A1" display="Case Study 1" xr:uid="{88CC4F86-7FA3-4145-B1B3-F5C38C42965F}"/>
@@ -4269,24 +4270,24 @@
       <c r="O3" s="19"/>
     </row>
     <row r="4" spans="1:15" ht="39" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="75" t="s">
+      <c r="A4" s="80" t="s">
         <v>176</v>
       </c>
-      <c r="B4" s="75"/>
-      <c r="C4" s="75"/>
-      <c r="D4" s="75"/>
-      <c r="E4" s="75"/>
-      <c r="F4" s="75"/>
+      <c r="B4" s="80"/>
+      <c r="C4" s="80"/>
+      <c r="D4" s="80"/>
+      <c r="E4" s="80"/>
+      <c r="F4" s="80"/>
     </row>
     <row r="5" spans="1:15" ht="38" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="75" t="s">
+      <c r="A5" s="80" t="s">
         <v>177</v>
       </c>
-      <c r="B5" s="75"/>
-      <c r="C5" s="75"/>
-      <c r="D5" s="75"/>
-      <c r="E5" s="75"/>
-      <c r="F5" s="75"/>
+      <c r="B5" s="80"/>
+      <c r="C5" s="80"/>
+      <c r="D5" s="80"/>
+      <c r="E5" s="80"/>
+      <c r="F5" s="80"/>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A6" s="40" t="s">
@@ -4334,32 +4335,32 @@
       <c r="K11" s="32"/>
     </row>
     <row r="12" spans="1:15" ht="24" x14ac:dyDescent="0.2">
-      <c r="A12" s="84" t="s">
+      <c r="A12" s="81" t="s">
         <v>35</v>
       </c>
-      <c r="B12" s="85"/>
-      <c r="C12" s="85"/>
-      <c r="D12" s="85"/>
-      <c r="E12" s="85"/>
-      <c r="F12" s="85"/>
-      <c r="G12" s="85"/>
-      <c r="H12" s="85"/>
-      <c r="I12" s="85"/>
-      <c r="J12" s="86"/>
+      <c r="B12" s="82"/>
+      <c r="C12" s="82"/>
+      <c r="D12" s="82"/>
+      <c r="E12" s="82"/>
+      <c r="F12" s="82"/>
+      <c r="G12" s="82"/>
+      <c r="H12" s="82"/>
+      <c r="I12" s="82"/>
+      <c r="J12" s="83"/>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A13" s="87" t="s">
+      <c r="A13" s="84" t="s">
         <v>36</v>
       </c>
-      <c r="B13" s="88"/>
-      <c r="C13" s="88"/>
-      <c r="D13" s="88"/>
-      <c r="E13" s="88"/>
-      <c r="F13" s="88"/>
-      <c r="G13" s="88"/>
-      <c r="H13" s="88"/>
-      <c r="I13" s="88"/>
-      <c r="J13" s="89"/>
+      <c r="B13" s="85"/>
+      <c r="C13" s="85"/>
+      <c r="D13" s="85"/>
+      <c r="E13" s="85"/>
+      <c r="F13" s="85"/>
+      <c r="G13" s="85"/>
+      <c r="H13" s="85"/>
+      <c r="I13" s="85"/>
+      <c r="J13" s="86"/>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A14" s="16" t="s">
@@ -4997,12 +4998,12 @@
       <c r="K57" s="32"/>
     </row>
     <row r="59" spans="1:11" ht="24" x14ac:dyDescent="0.2">
-      <c r="A59" s="83" t="s">
+      <c r="A59" s="87" t="s">
         <v>72</v>
       </c>
-      <c r="B59" s="83"/>
-      <c r="C59" s="83"/>
-      <c r="D59" s="83"/>
+      <c r="B59" s="87"/>
+      <c r="C59" s="87"/>
+      <c r="D59" s="87"/>
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A60" s="17" t="s">
@@ -5137,12 +5138,12 @@
       <c r="D89" s="78"/>
     </row>
     <row r="91" spans="1:5" ht="24" x14ac:dyDescent="0.2">
-      <c r="A91" s="83" t="s">
+      <c r="A91" s="87" t="s">
         <v>81</v>
       </c>
-      <c r="B91" s="83"/>
-      <c r="C91" s="83"/>
-      <c r="D91" s="83"/>
+      <c r="B91" s="87"/>
+      <c r="C91" s="87"/>
+      <c r="D91" s="87"/>
     </row>
     <row r="92" spans="1:5" ht="98" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A92" s="78" t="s">
@@ -5154,18 +5155,19 @@
       <c r="E92" s="13"/>
     </row>
   </sheetData>
+  <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="11">
-    <mergeCell ref="A4:F4"/>
-    <mergeCell ref="A5:F5"/>
-    <mergeCell ref="A12:J12"/>
-    <mergeCell ref="A13:J13"/>
-    <mergeCell ref="A65:D65"/>
     <mergeCell ref="A78:D78"/>
     <mergeCell ref="A89:D89"/>
     <mergeCell ref="A92:D92"/>
     <mergeCell ref="A91:D91"/>
     <mergeCell ref="A59:D59"/>
     <mergeCell ref="A70:D70"/>
+    <mergeCell ref="A4:F4"/>
+    <mergeCell ref="A5:F5"/>
+    <mergeCell ref="A12:J12"/>
+    <mergeCell ref="A13:J13"/>
+    <mergeCell ref="A65:D65"/>
   </mergeCells>
   <conditionalFormatting sqref="E45:E54">
     <cfRule type="containsText" dxfId="16" priority="1" operator="containsText" text="Low">
@@ -5242,25 +5244,25 @@
       </c>
     </row>
     <row r="6" spans="1:11" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="75" t="s">
+      <c r="A6" s="80" t="s">
         <v>172</v>
       </c>
-      <c r="B6" s="75"/>
-      <c r="C6" s="75"/>
+      <c r="B6" s="80"/>
+      <c r="C6" s="80"/>
     </row>
     <row r="7" spans="1:11" ht="51" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="75" t="s">
+      <c r="A7" s="80" t="s">
         <v>173</v>
       </c>
-      <c r="B7" s="75"/>
-      <c r="C7" s="75"/>
+      <c r="B7" s="80"/>
+      <c r="C7" s="80"/>
     </row>
     <row r="8" spans="1:11" ht="53" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="75" t="s">
+      <c r="A8" s="80" t="s">
         <v>174</v>
       </c>
-      <c r="B8" s="75"/>
-      <c r="C8" s="75"/>
+      <c r="B8" s="80"/>
+      <c r="C8" s="80"/>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
@@ -5561,10 +5563,10 @@
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A41" s="91" t="s">
+      <c r="A41" s="88" t="s">
         <v>102</v>
       </c>
-      <c r="B41" s="91"/>
+      <c r="B41" s="88"/>
     </row>
     <row r="44" spans="1:9" ht="22" x14ac:dyDescent="0.3">
       <c r="A44" s="39" t="s">
@@ -6020,14 +6022,14 @@
       <c r="G74" s="59" t="s">
         <v>139</v>
       </c>
-      <c r="R74" s="90"/>
-      <c r="S74" s="90"/>
-      <c r="T74" s="90"/>
-      <c r="U74" s="90"/>
-      <c r="V74" s="90"/>
-      <c r="W74" s="90"/>
-      <c r="X74" s="90"/>
-      <c r="Y74" s="90"/>
+      <c r="R74" s="89"/>
+      <c r="S74" s="89"/>
+      <c r="T74" s="89"/>
+      <c r="U74" s="89"/>
+      <c r="V74" s="89"/>
+      <c r="W74" s="89"/>
+      <c r="X74" s="89"/>
+      <c r="Y74" s="89"/>
     </row>
     <row r="75" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A75" s="60" t="s">
@@ -6070,14 +6072,14 @@
         <v>502</v>
       </c>
       <c r="G76" s="60"/>
-      <c r="R76" s="90"/>
-      <c r="S76" s="90"/>
-      <c r="T76" s="90"/>
-      <c r="U76" s="90"/>
-      <c r="V76" s="90"/>
-      <c r="W76" s="90"/>
-      <c r="X76" s="90"/>
-      <c r="Y76" s="90"/>
+      <c r="R76" s="89"/>
+      <c r="S76" s="89"/>
+      <c r="T76" s="89"/>
+      <c r="U76" s="89"/>
+      <c r="V76" s="89"/>
+      <c r="W76" s="89"/>
+      <c r="X76" s="89"/>
+      <c r="Y76" s="89"/>
     </row>
     <row r="77" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A77" s="60"/>
@@ -6136,11 +6138,11 @@
       <c r="K82" s="32"/>
     </row>
     <row r="83" spans="1:11" ht="24" x14ac:dyDescent="0.2">
-      <c r="A83" s="83" t="s">
+      <c r="A83" s="87" t="s">
         <v>136</v>
       </c>
-      <c r="B83" s="83"/>
-      <c r="C83" s="83"/>
+      <c r="B83" s="87"/>
+      <c r="C83" s="87"/>
     </row>
     <row r="84" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A84" s="17" t="s">
@@ -6177,6 +6179,7 @@
       <c r="H88" s="10"/>
     </row>
   </sheetData>
+  <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="9">
     <mergeCell ref="A88:C88"/>
     <mergeCell ref="A83:C83"/>
@@ -6255,17 +6258,17 @@
       </c>
     </row>
     <row r="5" spans="1:17" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="75" t="s">
+      <c r="A5" s="80" t="s">
         <v>180</v>
       </c>
-      <c r="B5" s="75"/>
+      <c r="B5" s="80"/>
       <c r="C5" s="23"/>
     </row>
     <row r="6" spans="1:17" ht="37" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="75" t="s">
+      <c r="A6" s="80" t="s">
         <v>181</v>
       </c>
-      <c r="B6" s="75"/>
+      <c r="B6" s="80"/>
       <c r="C6" s="23"/>
       <c r="Q6" s="1"/>
     </row>
@@ -6729,11 +6732,11 @@
       <c r="M75" s="32"/>
     </row>
     <row r="76" spans="1:13" ht="22" x14ac:dyDescent="0.2">
-      <c r="A76" s="77" t="s">
+      <c r="A76" s="90" t="s">
         <v>165</v>
       </c>
-      <c r="B76" s="77"/>
-      <c r="C76" s="77"/>
+      <c r="B76" s="90"/>
+      <c r="C76" s="90"/>
     </row>
     <row r="77" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A77" s="59" t="s">
@@ -6951,13 +6954,14 @@
       <c r="C101" s="47"/>
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A102" s="91" t="s">
+      <c r="A102" s="88" t="s">
         <v>506</v>
       </c>
-      <c r="B102" s="91"/>
-      <c r="C102" s="91"/>
+      <c r="B102" s="88"/>
+      <c r="C102" s="88"/>
     </row>
   </sheetData>
+  <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="5">
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="A6:B6"/>
@@ -7018,10 +7022,10 @@
       </c>
     </row>
     <row r="5" spans="1:12" ht="93" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="75" t="s">
+      <c r="A5" s="80" t="s">
         <v>206</v>
       </c>
-      <c r="B5" s="75"/>
+      <c r="B5" s="80"/>
       <c r="C5" s="23"/>
       <c r="D5" s="41" t="s">
         <v>507</v>
@@ -7785,10 +7789,10 @@
       <c r="G77" s="32"/>
     </row>
     <row r="78" spans="1:7" ht="22" x14ac:dyDescent="0.2">
-      <c r="A78" s="76" t="s">
+      <c r="A78" s="91" t="s">
         <v>480</v>
       </c>
-      <c r="B78" s="76"/>
+      <c r="B78" s="91"/>
     </row>
     <row r="79" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
@@ -7863,10 +7867,10 @@
       <c r="B93" s="78"/>
     </row>
     <row r="94" spans="1:4" ht="22" x14ac:dyDescent="0.2">
-      <c r="A94" s="77" t="s">
+      <c r="A94" s="90" t="s">
         <v>479</v>
       </c>
-      <c r="B94" s="77"/>
+      <c r="B94" s="90"/>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.2">
       <c r="D95" s="17"/>
@@ -7888,6 +7892,7 @@
       <c r="D102" s="10"/>
     </row>
   </sheetData>
+  <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="8">
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="A78:B78"/>
@@ -7967,28 +7972,28 @@
       </c>
     </row>
     <row r="6" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="75" t="s">
+      <c r="A6" s="80" t="s">
         <v>272</v>
       </c>
-      <c r="B6" s="75"/>
+      <c r="B6" s="80"/>
       <c r="E6" s="42" t="s">
         <v>277</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="39" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="75" t="s">
+      <c r="A7" s="80" t="s">
         <v>273</v>
       </c>
-      <c r="B7" s="75"/>
+      <c r="B7" s="80"/>
       <c r="E7" s="42" t="s">
         <v>278</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="47" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="75" t="s">
+      <c r="A8" s="80" t="s">
         <v>274</v>
       </c>
-      <c r="B8" s="75"/>
+      <c r="B8" s="80"/>
       <c r="E8" s="42" t="s">
         <v>279</v>
       </c>
@@ -8003,10 +8008,10 @@
       </c>
     </row>
     <row r="10" spans="1:8" ht="34" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="75" t="s">
+      <c r="A10" s="80" t="s">
         <v>276</v>
       </c>
-      <c r="B10" s="75"/>
+      <c r="B10" s="80"/>
       <c r="E10" s="40" t="s">
         <v>281</v>
       </c>
@@ -8580,10 +8585,10 @@
       <c r="H62" s="32"/>
     </row>
     <row r="63" spans="1:8" ht="22" x14ac:dyDescent="0.2">
-      <c r="A63" s="77" t="s">
+      <c r="A63" s="90" t="s">
         <v>481</v>
       </c>
-      <c r="B63" s="77"/>
+      <c r="B63" s="90"/>
     </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
@@ -8656,18 +8661,19 @@
       <c r="E93" s="10"/>
     </row>
   </sheetData>
+  <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="11">
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="A63:B63"/>
     <mergeCell ref="A72:B72"/>
     <mergeCell ref="A69:B69"/>
     <mergeCell ref="A66:B66"/>
     <mergeCell ref="A67:B67"/>
     <mergeCell ref="A70:B70"/>
     <mergeCell ref="A71:B71"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="A63:B63"/>
   </mergeCells>
   <conditionalFormatting sqref="F54:F59">
     <cfRule type="containsText" dxfId="7" priority="2" operator="containsText" text="additional">
@@ -8743,12 +8749,12 @@
       </c>
     </row>
     <row r="6" spans="1:13" ht="39" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="75" t="s">
+      <c r="A6" s="80" t="s">
         <v>314</v>
       </c>
-      <c r="B6" s="75"/>
-      <c r="C6" s="75"/>
-      <c r="D6" s="75"/>
+      <c r="B6" s="80"/>
+      <c r="C6" s="80"/>
+      <c r="D6" s="80"/>
       <c r="E6" s="23"/>
       <c r="G6" s="34" t="s">
         <v>318</v>
@@ -8756,12 +8762,12 @@
       <c r="H6" s="16"/>
     </row>
     <row r="7" spans="1:13" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="75" t="s">
+      <c r="A7" s="80" t="s">
         <v>317</v>
       </c>
-      <c r="B7" s="75"/>
-      <c r="C7" s="75"/>
-      <c r="D7" s="75"/>
+      <c r="B7" s="80"/>
+      <c r="C7" s="80"/>
+      <c r="D7" s="80"/>
       <c r="E7" s="23"/>
       <c r="F7" s="23"/>
       <c r="G7" t="s">
@@ -8769,20 +8775,20 @@
       </c>
     </row>
     <row r="8" spans="1:13" ht="57" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="75" t="s">
+      <c r="A8" s="80" t="s">
         <v>316</v>
       </c>
-      <c r="B8" s="75"/>
-      <c r="C8" s="75"/>
-      <c r="D8" s="75"/>
+      <c r="B8" s="80"/>
+      <c r="C8" s="80"/>
+      <c r="D8" s="80"/>
       <c r="E8" s="23"/>
       <c r="F8" s="23"/>
-      <c r="G8" s="75" t="s">
+      <c r="G8" s="80" t="s">
         <v>320</v>
       </c>
-      <c r="H8" s="75"/>
-      <c r="I8" s="75"/>
-      <c r="J8" s="75"/>
+      <c r="H8" s="80"/>
+      <c r="I8" s="80"/>
+      <c r="J8" s="80"/>
       <c r="K8" s="23"/>
       <c r="L8" s="23"/>
       <c r="M8" s="23"/>
@@ -9344,10 +9350,10 @@
       <c r="M68" s="32"/>
     </row>
     <row r="70" spans="1:13" ht="22" x14ac:dyDescent="0.2">
-      <c r="A70" s="77" t="s">
+      <c r="A70" s="90" t="s">
         <v>372</v>
       </c>
-      <c r="B70" s="77"/>
+      <c r="B70" s="90"/>
     </row>
     <row r="71" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
@@ -9397,15 +9403,16 @@
       <c r="A105" s="3"/>
     </row>
   </sheetData>
+  <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="8">
+    <mergeCell ref="G8:J8"/>
+    <mergeCell ref="A70:B70"/>
     <mergeCell ref="A74:B74"/>
     <mergeCell ref="A75:B75"/>
     <mergeCell ref="A76:B76"/>
     <mergeCell ref="A6:D6"/>
     <mergeCell ref="A7:D7"/>
     <mergeCell ref="A8:D8"/>
-    <mergeCell ref="G8:J8"/>
-    <mergeCell ref="A70:B70"/>
   </mergeCells>
   <conditionalFormatting sqref="C31">
     <cfRule type="expression" dxfId="5" priority="1">
@@ -9475,22 +9482,22 @@
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A6" s="75" t="s">
+      <c r="A6" s="80" t="s">
         <v>376</v>
       </c>
-      <c r="B6" s="75"/>
-      <c r="C6" s="75"/>
-      <c r="D6" s="75"/>
-      <c r="E6" s="75"/>
+      <c r="B6" s="80"/>
+      <c r="C6" s="80"/>
+      <c r="D6" s="80"/>
+      <c r="E6" s="80"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A7" s="75" t="s">
+      <c r="A7" s="80" t="s">
         <v>377</v>
       </c>
-      <c r="B7" s="75"/>
-      <c r="C7" s="75"/>
-      <c r="D7" s="75"/>
-      <c r="E7" s="75"/>
+      <c r="B7" s="80"/>
+      <c r="C7" s="80"/>
+      <c r="D7" s="80"/>
+      <c r="E7" s="80"/>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" s="40" t="s">
@@ -9502,22 +9509,22 @@
       <c r="E8" s="40"/>
     </row>
     <row r="9" spans="1:10" ht="35" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="75" t="s">
+      <c r="A9" s="80" t="s">
         <v>379</v>
       </c>
-      <c r="B9" s="75"/>
-      <c r="C9" s="75"/>
-      <c r="D9" s="75"/>
-      <c r="E9" s="75"/>
+      <c r="B9" s="80"/>
+      <c r="C9" s="80"/>
+      <c r="D9" s="80"/>
+      <c r="E9" s="80"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A10" s="75" t="s">
+      <c r="A10" s="80" t="s">
         <v>380</v>
       </c>
-      <c r="B10" s="75"/>
-      <c r="C10" s="75"/>
-      <c r="D10" s="75"/>
-      <c r="E10" s="75"/>
+      <c r="B10" s="80"/>
+      <c r="C10" s="80"/>
+      <c r="D10" s="80"/>
+      <c r="E10" s="80"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" s="40" t="s">
@@ -9529,13 +9536,13 @@
       <c r="E11" s="40"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A12" s="75" t="s">
+      <c r="A12" s="80" t="s">
         <v>382</v>
       </c>
-      <c r="B12" s="75"/>
-      <c r="C12" s="75"/>
-      <c r="D12" s="75"/>
-      <c r="E12" s="75"/>
+      <c r="B12" s="80"/>
+      <c r="C12" s="80"/>
+      <c r="D12" s="80"/>
+      <c r="E12" s="80"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
@@ -10312,10 +10319,10 @@
       <c r="J114" s="32"/>
     </row>
     <row r="115" spans="1:14" ht="24" x14ac:dyDescent="0.2">
-      <c r="A115" s="83" t="s">
+      <c r="A115" s="87" t="s">
         <v>73</v>
       </c>
-      <c r="B115" s="83"/>
+      <c r="B115" s="87"/>
       <c r="N115" s="10"/>
     </row>
     <row r="116" spans="1:14" ht="19" x14ac:dyDescent="0.25">
@@ -10358,10 +10365,10 @@
       <c r="B121" s="78"/>
     </row>
     <row r="123" spans="1:14" ht="24" x14ac:dyDescent="0.2">
-      <c r="A123" s="83" t="s">
+      <c r="A123" s="87" t="s">
         <v>374</v>
       </c>
-      <c r="B123" s="83"/>
+      <c r="B123" s="87"/>
     </row>
     <row r="124" spans="1:14" ht="19" x14ac:dyDescent="0.25">
       <c r="A124" s="6" t="s">
@@ -10397,12 +10404,8 @@
       <c r="B131" s="78"/>
     </row>
   </sheetData>
+  <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="13">
-    <mergeCell ref="A12:E12"/>
-    <mergeCell ref="A6:E6"/>
-    <mergeCell ref="A7:E7"/>
-    <mergeCell ref="A9:E9"/>
-    <mergeCell ref="A10:E10"/>
     <mergeCell ref="A131:B131"/>
     <mergeCell ref="A119:B119"/>
     <mergeCell ref="A120:B120"/>
@@ -10411,6 +10414,11 @@
     <mergeCell ref="A123:B123"/>
     <mergeCell ref="A125:B125"/>
     <mergeCell ref="A128:B128"/>
+    <mergeCell ref="A12:E12"/>
+    <mergeCell ref="A6:E6"/>
+    <mergeCell ref="A7:E7"/>
+    <mergeCell ref="A9:E9"/>
+    <mergeCell ref="A10:E10"/>
   </mergeCells>
   <conditionalFormatting sqref="E11:E106">
     <cfRule type="containsText" dxfId="3" priority="3" operator="containsText" text="Medium">

</xml_diff>

<commit_message>
Deploy updated case study workbook
Syncs gh-pages with master (commit 9c452b2).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/case-study/Cypress-Manufacturing-Payroll-Case-Study.xlsx
+++ b/assets/case-study/Cypress-Manufacturing-Payroll-Case-Study.xlsx
@@ -3,10 +3,10 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{477FDEDE-B894-5743-A9F4-0D923AEC60FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{958E5648-DFE6-DC4A-A98F-095A561D46F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="16060" xr2:uid="{C4273654-4867-1941-B027-2D844191C07C}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="16060" activeTab="7" xr2:uid="{C4273654-4867-1941-B027-2D844191C07C}"/>
   </bookViews>
   <sheets>
     <sheet name="Case Study Structure" sheetId="2" r:id="rId1"/>
@@ -2485,32 +2485,23 @@
     <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="27" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="6" fontId="10" fillId="5" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="25" fillId="4" borderId="0" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="17" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -2530,11 +2521,20 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -2935,6 +2935,51 @@
       </font>
     </dxf>
     <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="12" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="21" formatCode="d\-mmm"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="164" formatCode="0.0%"/>
     </dxf>
     <dxf>
@@ -3211,51 +3256,6 @@
         <bottom/>
       </border>
     </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="12" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="21" formatCode="d\-mmm"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -3270,7 +3270,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{383E5A6A-9EA9-DC47-B482-CE4D1C46D702}" name="Table1" displayName="Table1" ref="A5:D6" totalsRowShown="0" headerRowDxfId="70" headerRowBorderDxfId="69" tableBorderDxfId="68" totalsRowBorderDxfId="67">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{383E5A6A-9EA9-DC47-B482-CE4D1C46D702}" name="Table1" displayName="Table1" ref="A5:D6" totalsRowShown="0" headerRowDxfId="75" headerRowBorderDxfId="74" tableBorderDxfId="73" totalsRowBorderDxfId="72">
   <autoFilter ref="A5:D6" xr:uid="{383E5A6A-9EA9-DC47-B482-CE4D1C46D702}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -3278,10 +3278,10 @@
     <filterColumn colId="3" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{AEDF3CE8-2DEB-EE45-8C53-1F85628633A7}" name="Industry" dataDxfId="66"/>
-    <tableColumn id="2" xr3:uid="{0B994CEB-94AD-4140-97F8-CDD33306A830}" name="Software" dataDxfId="65"/>
-    <tableColumn id="3" xr3:uid="{65967071-3AC9-3942-AA02-B3F2B5DB301B}" name="Headquarters" dataDxfId="64"/>
-    <tableColumn id="4" xr3:uid="{1BD4C854-3956-9E49-957F-40F4FCA0FAD5}" name="Pay Frequency" dataDxfId="63"/>
+    <tableColumn id="1" xr3:uid="{AEDF3CE8-2DEB-EE45-8C53-1F85628633A7}" name="Industry" dataDxfId="71"/>
+    <tableColumn id="2" xr3:uid="{0B994CEB-94AD-4140-97F8-CDD33306A830}" name="Software" dataDxfId="70"/>
+    <tableColumn id="3" xr3:uid="{65967071-3AC9-3942-AA02-B3F2B5DB301B}" name="Headquarters" dataDxfId="69"/>
+    <tableColumn id="4" xr3:uid="{1BD4C854-3956-9E49-957F-40F4FCA0FAD5}" name="Pay Frequency" dataDxfId="68"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium20" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3394,7 +3394,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{6FE775DD-B461-4347-8D3F-819C8C31609A}" name="Table2" displayName="Table2" ref="A14:J24" totalsRowShown="0" headerRowDxfId="62">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{6FE775DD-B461-4347-8D3F-819C8C31609A}" name="Table2" displayName="Table2" ref="A14:J24" totalsRowShown="0" headerRowDxfId="67">
   <autoFilter ref="A14:J24" xr:uid="{6FE775DD-B461-4347-8D3F-819C8C31609A}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -3416,15 +3416,15 @@
     <tableColumn id="6" xr3:uid="{224D6D44-F303-774C-A528-92B3AA22879B}" name="Pay Type"/>
     <tableColumn id="7" xr3:uid="{868140BC-A833-124B-A94F-8B5A38DEF6A5}" name="Regular Hours"/>
     <tableColumn id="8" xr3:uid="{E671470B-0A1C-874B-A4AA-533A39A3CFA8}" name="OT Hours"/>
-    <tableColumn id="9" xr3:uid="{950491E5-BEFA-CA4D-A832-6FE31057E0B7}" name="Hourly Rate" dataDxfId="61"/>
-    <tableColumn id="10" xr3:uid="{680896A4-4C9A-0F48-AACB-EA763B9AB3A2}" name="Gross Pay" dataDxfId="60"/>
+    <tableColumn id="9" xr3:uid="{950491E5-BEFA-CA4D-A832-6FE31057E0B7}" name="Hourly Rate" dataDxfId="66"/>
+    <tableColumn id="10" xr3:uid="{680896A4-4C9A-0F48-AACB-EA763B9AB3A2}" name="Gross Pay" dataDxfId="65"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium6" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{2A7F74B7-2140-0943-A44D-A7F630110CEF}" name="Table3" displayName="Table3" ref="A44:E54" totalsRowShown="0" headerRowDxfId="59" dataDxfId="57" headerRowBorderDxfId="58" tableBorderDxfId="56">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{2A7F74B7-2140-0943-A44D-A7F630110CEF}" name="Table3" displayName="Table3" ref="A44:E54" totalsRowShown="0" headerRowDxfId="64" dataDxfId="62" headerRowBorderDxfId="63" tableBorderDxfId="61">
   <autoFilter ref="A44:E54" xr:uid="{2A7F74B7-2140-0943-A44D-A7F630110CEF}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -3434,9 +3434,9 @@
   </autoFilter>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{F501A1CD-2634-1E45-B325-ED46A02A8C59}" name="Employee"/>
-    <tableColumn id="2" xr3:uid="{094C7B36-23E9-2D46-A3B4-89252F172225}" name="Observation" dataDxfId="55"/>
-    <tableColumn id="3" xr3:uid="{D96B0134-ADDF-A34C-A43B-70661D422E93}" name="Why It Matters" dataDxfId="54"/>
-    <tableColumn id="4" xr3:uid="{A8571B47-41AC-0A43-A0AF-72A79C41C66E}" name="Recommended Next Step" dataDxfId="53"/>
+    <tableColumn id="2" xr3:uid="{094C7B36-23E9-2D46-A3B4-89252F172225}" name="Observation" dataDxfId="60"/>
+    <tableColumn id="3" xr3:uid="{D96B0134-ADDF-A34C-A43B-70661D422E93}" name="Why It Matters" dataDxfId="59"/>
+    <tableColumn id="4" xr3:uid="{A8571B47-41AC-0A43-A0AF-72A79C41C66E}" name="Recommended Next Step" dataDxfId="58"/>
     <tableColumn id="5" xr3:uid="{2592205F-EC3A-0546-A69E-71189210BB12}" name="Priority"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium6" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -3444,7 +3444,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{351AEDD7-0B28-4149-813B-66FA9F159C6C}" name="Table4" displayName="Table4" ref="A16:F23" totalsRowShown="0" headerRowDxfId="52">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{351AEDD7-0B28-4149-813B-66FA9F159C6C}" name="Table4" displayName="Table4" ref="A16:F23" totalsRowShown="0" headerRowDxfId="57">
   <autoFilter ref="A16:F23" xr:uid="{351AEDD7-0B28-4149-813B-66FA9F159C6C}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -3458,15 +3458,15 @@
     <tableColumn id="2" xr3:uid="{028E131D-1589-154E-A6BC-D933B354CFCA}" name="Previous OT Hours"/>
     <tableColumn id="3" xr3:uid="{B62BADED-F710-404F-82FD-857F0A99A4C2}" name="Current OT Hours"/>
     <tableColumn id="4" xr3:uid="{AF395F61-6C52-6C48-B882-4C60B174C066}" name="Change"/>
-    <tableColumn id="5" xr3:uid="{1A5D0D21-0C3C-5846-8142-100D11DE10BC}" name="Previous OT Cost" dataDxfId="51"/>
-    <tableColumn id="6" xr3:uid="{445B8E35-D644-904D-A104-13802A5197F3}" name="Current OT Cost" dataDxfId="50"/>
+    <tableColumn id="5" xr3:uid="{1A5D0D21-0C3C-5846-8142-100D11DE10BC}" name="Previous OT Cost" dataDxfId="56"/>
+    <tableColumn id="6" xr3:uid="{445B8E35-D644-904D-A104-13802A5197F3}" name="Current OT Cost" dataDxfId="55"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium6" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{0EF008CC-394B-6344-AF94-A7DCA1F43A7B}" name="Table5" displayName="Table5" ref="A63:K71" totalsRowShown="0" headerRowDxfId="49">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{0EF008CC-394B-6344-AF94-A7DCA1F43A7B}" name="Table5" displayName="Table5" ref="A63:K71" totalsRowShown="0" headerRowDxfId="54">
   <autoFilter ref="A63:K71" xr:uid="{0EF008CC-394B-6344-AF94-A7DCA1F43A7B}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -3485,12 +3485,12 @@
     <tableColumn id="2" xr3:uid="{D1DFEE06-891B-0A43-AB23-F4B8B17E8764}" name="Previous OT Hours"/>
     <tableColumn id="3" xr3:uid="{E07B0018-BC29-DD48-93E8-A71A47034A50}" name="Current OT Hours"/>
     <tableColumn id="4" xr3:uid="{D3727CA9-7D49-1648-8211-1BD086564169}" name="OT Variance"/>
-    <tableColumn id="5" xr3:uid="{0F4DF983-C252-1E4E-B5A2-FF2561B38668}" name="% Change/Increase (Hours)" dataDxfId="48" dataCellStyle="Percent"/>
-    <tableColumn id="6" xr3:uid="{37F4AE63-1CD6-EF4C-9115-9FD3C30C84F3}" name="Previous OT Cost" dataDxfId="47"/>
-    <tableColumn id="7" xr3:uid="{D1F9C495-D850-CB48-916B-84D9499A9448}" name="Current OT Cost" dataDxfId="46"/>
-    <tableColumn id="8" xr3:uid="{03A9D69E-29BB-624F-84D0-A5DFE8B0A3A3}" name="OT Cost Variance" dataDxfId="45"/>
-    <tableColumn id="9" xr3:uid="{4B69023F-FD00-D140-AFDE-B6E3A801B121}" name="% Change/Increase (Cost)" dataDxfId="44" dataCellStyle="Percent"/>
-    <tableColumn id="10" xr3:uid="{0C1A6056-F07A-8340-AC97-8AB86E910DC5}" name="Contribution to Total Increase" dataDxfId="43"/>
+    <tableColumn id="5" xr3:uid="{0F4DF983-C252-1E4E-B5A2-FF2561B38668}" name="% Change/Increase (Hours)" dataDxfId="53" dataCellStyle="Percent"/>
+    <tableColumn id="6" xr3:uid="{37F4AE63-1CD6-EF4C-9115-9FD3C30C84F3}" name="Previous OT Cost" dataDxfId="52"/>
+    <tableColumn id="7" xr3:uid="{D1F9C495-D850-CB48-916B-84D9499A9448}" name="Current OT Cost" dataDxfId="51"/>
+    <tableColumn id="8" xr3:uid="{03A9D69E-29BB-624F-84D0-A5DFE8B0A3A3}" name="OT Cost Variance" dataDxfId="50"/>
+    <tableColumn id="9" xr3:uid="{4B69023F-FD00-D140-AFDE-B6E3A801B121}" name="% Change/Increase (Cost)" dataDxfId="49" dataCellStyle="Percent"/>
+    <tableColumn id="10" xr3:uid="{0C1A6056-F07A-8340-AC97-8AB86E910DC5}" name="Contribution to Total Increase" dataDxfId="48"/>
     <tableColumn id="11" xr3:uid="{9A38B402-FD83-5249-80A6-81FFB1FDEDE2}" name="Notes"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium6" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -3498,7 +3498,7 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{94DD0E59-552A-004A-AE6C-3461962A0666}" name="Table6" displayName="Table6" ref="A18:G28" totalsRowShown="0" headerRowDxfId="75">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{94DD0E59-552A-004A-AE6C-3461962A0666}" name="Table6" displayName="Table6" ref="A18:G28" totalsRowShown="0" headerRowDxfId="47">
   <autoFilter ref="A18:G28" xr:uid="{94DD0E59-552A-004A-AE6C-3461962A0666}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -3511,7 +3511,7 @@
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{6E7464B2-2E9D-BC4B-BACE-FCCA89663E10}" name="Employee"/>
     <tableColumn id="2" xr3:uid="{6E0AF0A4-5FBE-FA40-96D1-32AE0AAB9F99}" name="Department"/>
-    <tableColumn id="3" xr3:uid="{6BAB4C3B-FB41-604B-8388-79605B985199}" name="Date" dataDxfId="74"/>
+    <tableColumn id="3" xr3:uid="{6BAB4C3B-FB41-604B-8388-79605B985199}" name="Date" dataDxfId="46"/>
     <tableColumn id="4" xr3:uid="{D0A68926-DC3B-074D-9592-84E6C512199E}" name="Shift Hours"/>
     <tableColumn id="5" xr3:uid="{76E90D76-F085-4F48-AE39-8EE88D5C33DA}" name="Meal Break"/>
     <tableColumn id="6" xr3:uid="{FA9160F9-C4F5-2243-BE46-63983AABFEA4}" name="Premium Paid"/>
@@ -3522,7 +3522,7 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{40F5E122-6DFE-6045-8A75-1C80ACE768C1}" name="Table7" displayName="Table7" ref="A63:F74" totalsRowShown="0" headerRowDxfId="73">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{40F5E122-6DFE-6045-8A75-1C80ACE768C1}" name="Table7" displayName="Table7" ref="A63:F74" totalsRowShown="0" headerRowDxfId="45">
   <autoFilter ref="A63:F74" xr:uid="{40F5E122-6DFE-6045-8A75-1C80ACE768C1}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -3536,8 +3536,8 @@
     <tableColumn id="2" xr3:uid="{8379B859-ADC9-0A45-9488-7A8D98D4FE19}" name="Exception"/>
     <tableColumn id="3" xr3:uid="{B5FFCA04-440B-5044-A809-AD21B4512853}" name="Evidence"/>
     <tableColumn id="4" xr3:uid="{D20F569C-B6FC-774E-8651-D3A95806B131}" name="Does It Require Review?"/>
-    <tableColumn id="5" xr3:uid="{388A88A7-6C48-B64D-A56E-A50F28A25F64}" name="Potential Premium" dataDxfId="72"/>
-    <tableColumn id="6" xr3:uid="{30ACDD88-9666-3F40-BD0E-7CF6A6A94BFE}" name="Questions" dataDxfId="71"/>
+    <tableColumn id="5" xr3:uid="{388A88A7-6C48-B64D-A56E-A50F28A25F64}" name="Potential Premium" dataDxfId="44"/>
+    <tableColumn id="6" xr3:uid="{30ACDD88-9666-3F40-BD0E-7CF6A6A94BFE}" name="Questions" dataDxfId="43"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium6" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3938,10 +3938,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="32" x14ac:dyDescent="0.4">
-      <c r="A1" s="82" t="s">
+      <c r="A1" s="77" t="s">
         <v>42</v>
       </c>
-      <c r="B1" s="82"/>
+      <c r="B1" s="77"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="78" t="s">
@@ -3988,20 +3988,20 @@
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A8" s="79" t="s">
+      <c r="A8" s="75" t="s">
         <v>483</v>
       </c>
-      <c r="B8" s="79"/>
-      <c r="C8" s="79"/>
-      <c r="D8" s="79"/>
+      <c r="B8" s="75"/>
+      <c r="C8" s="75"/>
+      <c r="D8" s="75"/>
     </row>
     <row r="9" spans="1:6" ht="27" x14ac:dyDescent="0.2">
-      <c r="A9" s="81" t="s">
+      <c r="A9" s="79" t="s">
         <v>529</v>
       </c>
-      <c r="B9" s="81"/>
-      <c r="C9" s="81"/>
-      <c r="D9" s="81"/>
+      <c r="B9" s="79"/>
+      <c r="C9" s="79"/>
+      <c r="D9" s="79"/>
     </row>
     <row r="10" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="78" t="s">
@@ -4015,20 +4015,20 @@
       <c r="A11" s="17"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A12" s="79" t="s">
+      <c r="A12" s="75" t="s">
         <v>484</v>
       </c>
-      <c r="B12" s="79"/>
-      <c r="C12" s="79"/>
-      <c r="D12" s="79"/>
+      <c r="B12" s="75"/>
+      <c r="C12" s="75"/>
+      <c r="D12" s="75"/>
     </row>
     <row r="13" spans="1:6" ht="27" x14ac:dyDescent="0.2">
-      <c r="A13" s="81" t="s">
+      <c r="A13" s="79" t="s">
         <v>530</v>
       </c>
-      <c r="B13" s="81"/>
-      <c r="C13" s="81"/>
-      <c r="D13" s="81"/>
+      <c r="B13" s="79"/>
+      <c r="C13" s="79"/>
+      <c r="D13" s="79"/>
     </row>
     <row r="14" spans="1:6" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="78" t="s">
@@ -4042,130 +4042,130 @@
       <c r="A15" s="17"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A16" s="79" t="s">
+      <c r="A16" s="75" t="s">
         <v>485</v>
       </c>
-      <c r="B16" s="79"/>
-      <c r="C16" s="79"/>
-      <c r="D16" s="79"/>
+      <c r="B16" s="75"/>
+      <c r="C16" s="75"/>
+      <c r="D16" s="75"/>
     </row>
     <row r="17" spans="1:4" ht="27" x14ac:dyDescent="0.2">
-      <c r="A17" s="81" t="s">
+      <c r="A17" s="79" t="s">
         <v>531</v>
       </c>
-      <c r="B17" s="81"/>
-      <c r="C17" s="81"/>
-      <c r="D17" s="81"/>
+      <c r="B17" s="79"/>
+      <c r="C17" s="79"/>
+      <c r="D17" s="79"/>
     </row>
     <row r="18" spans="1:4" ht="35" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="80" t="s">
+      <c r="A18" s="76" t="s">
         <v>473</v>
       </c>
-      <c r="B18" s="80"/>
-      <c r="C18" s="80"/>
-      <c r="D18" s="80"/>
+      <c r="B18" s="76"/>
+      <c r="C18" s="76"/>
+      <c r="D18" s="76"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" s="1"/>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A20" s="79" t="s">
+      <c r="A20" s="75" t="s">
         <v>486</v>
       </c>
-      <c r="B20" s="79"/>
-      <c r="C20" s="79"/>
-      <c r="D20" s="79"/>
+      <c r="B20" s="75"/>
+      <c r="C20" s="75"/>
+      <c r="D20" s="75"/>
     </row>
     <row r="21" spans="1:4" ht="27" x14ac:dyDescent="0.2">
-      <c r="A21" s="81" t="s">
+      <c r="A21" s="79" t="s">
         <v>532</v>
       </c>
-      <c r="B21" s="81"/>
-      <c r="C21" s="81"/>
-      <c r="D21" s="81"/>
+      <c r="B21" s="79"/>
+      <c r="C21" s="79"/>
+      <c r="D21" s="79"/>
     </row>
     <row r="22" spans="1:4" ht="34" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="80" t="s">
+      <c r="A22" s="76" t="s">
         <v>474</v>
       </c>
-      <c r="B22" s="80"/>
-      <c r="C22" s="80"/>
-      <c r="D22" s="80"/>
+      <c r="B22" s="76"/>
+      <c r="C22" s="76"/>
+      <c r="D22" s="76"/>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A24" s="79" t="s">
+      <c r="A24" s="75" t="s">
         <v>487</v>
       </c>
-      <c r="B24" s="79"/>
-      <c r="C24" s="79"/>
-      <c r="D24" s="79"/>
+      <c r="B24" s="75"/>
+      <c r="C24" s="75"/>
+      <c r="D24" s="75"/>
     </row>
     <row r="25" spans="1:4" ht="27" x14ac:dyDescent="0.2">
-      <c r="A25" s="81" t="s">
+      <c r="A25" s="79" t="s">
         <v>533</v>
       </c>
-      <c r="B25" s="81"/>
-      <c r="C25" s="81"/>
-      <c r="D25" s="81"/>
+      <c r="B25" s="79"/>
+      <c r="C25" s="79"/>
+      <c r="D25" s="79"/>
     </row>
     <row r="26" spans="1:4" ht="35" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="80" t="s">
+      <c r="A26" s="76" t="s">
         <v>475</v>
       </c>
-      <c r="B26" s="80"/>
-      <c r="C26" s="80"/>
-      <c r="D26" s="80"/>
+      <c r="B26" s="76"/>
+      <c r="C26" s="76"/>
+      <c r="D26" s="76"/>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A27" s="1"/>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A28" s="79" t="s">
+      <c r="A28" s="75" t="s">
         <v>488</v>
       </c>
-      <c r="B28" s="79"/>
-      <c r="C28" s="79"/>
-      <c r="D28" s="79"/>
+      <c r="B28" s="75"/>
+      <c r="C28" s="75"/>
+      <c r="D28" s="75"/>
     </row>
     <row r="29" spans="1:4" ht="27" x14ac:dyDescent="0.2">
-      <c r="A29" s="81" t="s">
+      <c r="A29" s="79" t="s">
         <v>534</v>
       </c>
-      <c r="B29" s="81"/>
-      <c r="C29" s="81"/>
-      <c r="D29" s="81"/>
+      <c r="B29" s="79"/>
+      <c r="C29" s="79"/>
+      <c r="D29" s="79"/>
     </row>
     <row r="30" spans="1:4" ht="38" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="80" t="s">
+      <c r="A30" s="76" t="s">
         <v>493</v>
       </c>
-      <c r="B30" s="80"/>
-      <c r="C30" s="80"/>
-      <c r="D30" s="80"/>
+      <c r="B30" s="76"/>
+      <c r="C30" s="76"/>
+      <c r="D30" s="76"/>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A32" s="79" t="s">
+      <c r="A32" s="75" t="s">
         <v>489</v>
       </c>
-      <c r="B32" s="79"/>
-      <c r="C32" s="79"/>
-      <c r="D32" s="79"/>
+      <c r="B32" s="75"/>
+      <c r="C32" s="75"/>
+      <c r="D32" s="75"/>
     </row>
     <row r="33" spans="1:5" ht="27" x14ac:dyDescent="0.2">
-      <c r="A33" s="81" t="s">
+      <c r="A33" s="79" t="s">
         <v>373</v>
       </c>
-      <c r="B33" s="81"/>
-      <c r="C33" s="81"/>
-      <c r="D33" s="81"/>
+      <c r="B33" s="79"/>
+      <c r="C33" s="79"/>
+      <c r="D33" s="79"/>
     </row>
     <row r="34" spans="1:5" ht="37" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="80" t="s">
+      <c r="A34" s="76" t="s">
         <v>494</v>
       </c>
-      <c r="B34" s="80"/>
-      <c r="C34" s="80"/>
-      <c r="D34" s="80"/>
+      <c r="B34" s="76"/>
+      <c r="C34" s="76"/>
+      <c r="D34" s="76"/>
     </row>
     <row r="35" spans="1:5" ht="19" x14ac:dyDescent="0.25">
       <c r="C35" s="31"/>
@@ -4183,14 +4183,8 @@
       <c r="E37" s="1"/>
     </row>
   </sheetData>
+  <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="23">
-    <mergeCell ref="A20:D20"/>
-    <mergeCell ref="A22:D22"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A8:D8"/>
-    <mergeCell ref="A10:D10"/>
-    <mergeCell ref="A12:D12"/>
-    <mergeCell ref="A14:D14"/>
     <mergeCell ref="A32:D32"/>
     <mergeCell ref="A34:D34"/>
     <mergeCell ref="A2:C2"/>
@@ -4207,6 +4201,13 @@
     <mergeCell ref="A28:D28"/>
     <mergeCell ref="A30:D30"/>
     <mergeCell ref="A18:D18"/>
+    <mergeCell ref="A20:D20"/>
+    <mergeCell ref="A22:D22"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A8:D8"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="A12:D12"/>
+    <mergeCell ref="A14:D14"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A8:D8" location="'Monday Morning Payroll Week 1'!A1" display="Case Study 1" xr:uid="{88CC4F86-7FA3-4145-B1B3-F5C38C42965F}"/>
@@ -4269,24 +4270,24 @@
       <c r="O3" s="19"/>
     </row>
     <row r="4" spans="1:15" ht="39" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="75" t="s">
+      <c r="A4" s="80" t="s">
         <v>176</v>
       </c>
-      <c r="B4" s="75"/>
-      <c r="C4" s="75"/>
-      <c r="D4" s="75"/>
-      <c r="E4" s="75"/>
-      <c r="F4" s="75"/>
+      <c r="B4" s="80"/>
+      <c r="C4" s="80"/>
+      <c r="D4" s="80"/>
+      <c r="E4" s="80"/>
+      <c r="F4" s="80"/>
     </row>
     <row r="5" spans="1:15" ht="38" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="75" t="s">
+      <c r="A5" s="80" t="s">
         <v>177</v>
       </c>
-      <c r="B5" s="75"/>
-      <c r="C5" s="75"/>
-      <c r="D5" s="75"/>
-      <c r="E5" s="75"/>
-      <c r="F5" s="75"/>
+      <c r="B5" s="80"/>
+      <c r="C5" s="80"/>
+      <c r="D5" s="80"/>
+      <c r="E5" s="80"/>
+      <c r="F5" s="80"/>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A6" s="40" t="s">
@@ -4334,32 +4335,32 @@
       <c r="K11" s="32"/>
     </row>
     <row r="12" spans="1:15" ht="24" x14ac:dyDescent="0.2">
-      <c r="A12" s="84" t="s">
+      <c r="A12" s="81" t="s">
         <v>35</v>
       </c>
-      <c r="B12" s="85"/>
-      <c r="C12" s="85"/>
-      <c r="D12" s="85"/>
-      <c r="E12" s="85"/>
-      <c r="F12" s="85"/>
-      <c r="G12" s="85"/>
-      <c r="H12" s="85"/>
-      <c r="I12" s="85"/>
-      <c r="J12" s="86"/>
+      <c r="B12" s="82"/>
+      <c r="C12" s="82"/>
+      <c r="D12" s="82"/>
+      <c r="E12" s="82"/>
+      <c r="F12" s="82"/>
+      <c r="G12" s="82"/>
+      <c r="H12" s="82"/>
+      <c r="I12" s="82"/>
+      <c r="J12" s="83"/>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A13" s="87" t="s">
+      <c r="A13" s="84" t="s">
         <v>36</v>
       </c>
-      <c r="B13" s="88"/>
-      <c r="C13" s="88"/>
-      <c r="D13" s="88"/>
-      <c r="E13" s="88"/>
-      <c r="F13" s="88"/>
-      <c r="G13" s="88"/>
-      <c r="H13" s="88"/>
-      <c r="I13" s="88"/>
-      <c r="J13" s="89"/>
+      <c r="B13" s="85"/>
+      <c r="C13" s="85"/>
+      <c r="D13" s="85"/>
+      <c r="E13" s="85"/>
+      <c r="F13" s="85"/>
+      <c r="G13" s="85"/>
+      <c r="H13" s="85"/>
+      <c r="I13" s="85"/>
+      <c r="J13" s="86"/>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A14" s="16" t="s">
@@ -4997,12 +4998,12 @@
       <c r="K57" s="32"/>
     </row>
     <row r="59" spans="1:11" ht="24" x14ac:dyDescent="0.2">
-      <c r="A59" s="83" t="s">
+      <c r="A59" s="87" t="s">
         <v>72</v>
       </c>
-      <c r="B59" s="83"/>
-      <c r="C59" s="83"/>
-      <c r="D59" s="83"/>
+      <c r="B59" s="87"/>
+      <c r="C59" s="87"/>
+      <c r="D59" s="87"/>
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A60" s="17" t="s">
@@ -5137,12 +5138,12 @@
       <c r="D89" s="78"/>
     </row>
     <row r="91" spans="1:5" ht="24" x14ac:dyDescent="0.2">
-      <c r="A91" s="83" t="s">
+      <c r="A91" s="87" t="s">
         <v>81</v>
       </c>
-      <c r="B91" s="83"/>
-      <c r="C91" s="83"/>
-      <c r="D91" s="83"/>
+      <c r="B91" s="87"/>
+      <c r="C91" s="87"/>
+      <c r="D91" s="87"/>
     </row>
     <row r="92" spans="1:5" ht="98" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A92" s="78" t="s">
@@ -5154,18 +5155,19 @@
       <c r="E92" s="13"/>
     </row>
   </sheetData>
+  <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="11">
-    <mergeCell ref="A4:F4"/>
-    <mergeCell ref="A5:F5"/>
-    <mergeCell ref="A12:J12"/>
-    <mergeCell ref="A13:J13"/>
-    <mergeCell ref="A65:D65"/>
     <mergeCell ref="A78:D78"/>
     <mergeCell ref="A89:D89"/>
     <mergeCell ref="A92:D92"/>
     <mergeCell ref="A91:D91"/>
     <mergeCell ref="A59:D59"/>
     <mergeCell ref="A70:D70"/>
+    <mergeCell ref="A4:F4"/>
+    <mergeCell ref="A5:F5"/>
+    <mergeCell ref="A12:J12"/>
+    <mergeCell ref="A13:J13"/>
+    <mergeCell ref="A65:D65"/>
   </mergeCells>
   <conditionalFormatting sqref="E45:E54">
     <cfRule type="containsText" dxfId="16" priority="1" operator="containsText" text="Low">
@@ -5242,25 +5244,25 @@
       </c>
     </row>
     <row r="6" spans="1:11" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="75" t="s">
+      <c r="A6" s="80" t="s">
         <v>172</v>
       </c>
-      <c r="B6" s="75"/>
-      <c r="C6" s="75"/>
+      <c r="B6" s="80"/>
+      <c r="C6" s="80"/>
     </row>
     <row r="7" spans="1:11" ht="51" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="75" t="s">
+      <c r="A7" s="80" t="s">
         <v>173</v>
       </c>
-      <c r="B7" s="75"/>
-      <c r="C7" s="75"/>
+      <c r="B7" s="80"/>
+      <c r="C7" s="80"/>
     </row>
     <row r="8" spans="1:11" ht="53" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="75" t="s">
+      <c r="A8" s="80" t="s">
         <v>174</v>
       </c>
-      <c r="B8" s="75"/>
-      <c r="C8" s="75"/>
+      <c r="B8" s="80"/>
+      <c r="C8" s="80"/>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
@@ -5561,10 +5563,10 @@
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A41" s="91" t="s">
+      <c r="A41" s="88" t="s">
         <v>102</v>
       </c>
-      <c r="B41" s="91"/>
+      <c r="B41" s="88"/>
     </row>
     <row r="44" spans="1:9" ht="22" x14ac:dyDescent="0.3">
       <c r="A44" s="39" t="s">
@@ -6020,14 +6022,14 @@
       <c r="G74" s="59" t="s">
         <v>139</v>
       </c>
-      <c r="R74" s="90"/>
-      <c r="S74" s="90"/>
-      <c r="T74" s="90"/>
-      <c r="U74" s="90"/>
-      <c r="V74" s="90"/>
-      <c r="W74" s="90"/>
-      <c r="X74" s="90"/>
-      <c r="Y74" s="90"/>
+      <c r="R74" s="89"/>
+      <c r="S74" s="89"/>
+      <c r="T74" s="89"/>
+      <c r="U74" s="89"/>
+      <c r="V74" s="89"/>
+      <c r="W74" s="89"/>
+      <c r="X74" s="89"/>
+      <c r="Y74" s="89"/>
     </row>
     <row r="75" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A75" s="60" t="s">
@@ -6070,14 +6072,14 @@
         <v>502</v>
       </c>
       <c r="G76" s="60"/>
-      <c r="R76" s="90"/>
-      <c r="S76" s="90"/>
-      <c r="T76" s="90"/>
-      <c r="U76" s="90"/>
-      <c r="V76" s="90"/>
-      <c r="W76" s="90"/>
-      <c r="X76" s="90"/>
-      <c r="Y76" s="90"/>
+      <c r="R76" s="89"/>
+      <c r="S76" s="89"/>
+      <c r="T76" s="89"/>
+      <c r="U76" s="89"/>
+      <c r="V76" s="89"/>
+      <c r="W76" s="89"/>
+      <c r="X76" s="89"/>
+      <c r="Y76" s="89"/>
     </row>
     <row r="77" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A77" s="60"/>
@@ -6136,11 +6138,11 @@
       <c r="K82" s="32"/>
     </row>
     <row r="83" spans="1:11" ht="24" x14ac:dyDescent="0.2">
-      <c r="A83" s="83" t="s">
+      <c r="A83" s="87" t="s">
         <v>136</v>
       </c>
-      <c r="B83" s="83"/>
-      <c r="C83" s="83"/>
+      <c r="B83" s="87"/>
+      <c r="C83" s="87"/>
     </row>
     <row r="84" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A84" s="17" t="s">
@@ -6177,6 +6179,7 @@
       <c r="H88" s="10"/>
     </row>
   </sheetData>
+  <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="9">
     <mergeCell ref="A88:C88"/>
     <mergeCell ref="A83:C83"/>
@@ -6255,17 +6258,17 @@
       </c>
     </row>
     <row r="5" spans="1:17" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="75" t="s">
+      <c r="A5" s="80" t="s">
         <v>180</v>
       </c>
-      <c r="B5" s="75"/>
+      <c r="B5" s="80"/>
       <c r="C5" s="23"/>
     </row>
     <row r="6" spans="1:17" ht="37" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="75" t="s">
+      <c r="A6" s="80" t="s">
         <v>181</v>
       </c>
-      <c r="B6" s="75"/>
+      <c r="B6" s="80"/>
       <c r="C6" s="23"/>
       <c r="Q6" s="1"/>
     </row>
@@ -6729,11 +6732,11 @@
       <c r="M75" s="32"/>
     </row>
     <row r="76" spans="1:13" ht="22" x14ac:dyDescent="0.2">
-      <c r="A76" s="77" t="s">
+      <c r="A76" s="90" t="s">
         <v>165</v>
       </c>
-      <c r="B76" s="77"/>
-      <c r="C76" s="77"/>
+      <c r="B76" s="90"/>
+      <c r="C76" s="90"/>
     </row>
     <row r="77" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A77" s="59" t="s">
@@ -6951,13 +6954,14 @@
       <c r="C101" s="47"/>
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A102" s="91" t="s">
+      <c r="A102" s="88" t="s">
         <v>506</v>
       </c>
-      <c r="B102" s="91"/>
-      <c r="C102" s="91"/>
+      <c r="B102" s="88"/>
+      <c r="C102" s="88"/>
     </row>
   </sheetData>
+  <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="5">
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="A6:B6"/>
@@ -7018,10 +7022,10 @@
       </c>
     </row>
     <row r="5" spans="1:12" ht="93" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="75" t="s">
+      <c r="A5" s="80" t="s">
         <v>206</v>
       </c>
-      <c r="B5" s="75"/>
+      <c r="B5" s="80"/>
       <c r="C5" s="23"/>
       <c r="D5" s="41" t="s">
         <v>507</v>
@@ -7785,10 +7789,10 @@
       <c r="G77" s="32"/>
     </row>
     <row r="78" spans="1:7" ht="22" x14ac:dyDescent="0.2">
-      <c r="A78" s="76" t="s">
+      <c r="A78" s="91" t="s">
         <v>480</v>
       </c>
-      <c r="B78" s="76"/>
+      <c r="B78" s="91"/>
     </row>
     <row r="79" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
@@ -7863,10 +7867,10 @@
       <c r="B93" s="78"/>
     </row>
     <row r="94" spans="1:4" ht="22" x14ac:dyDescent="0.2">
-      <c r="A94" s="77" t="s">
+      <c r="A94" s="90" t="s">
         <v>479</v>
       </c>
-      <c r="B94" s="77"/>
+      <c r="B94" s="90"/>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.2">
       <c r="D95" s="17"/>
@@ -7888,6 +7892,7 @@
       <c r="D102" s="10"/>
     </row>
   </sheetData>
+  <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="8">
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="A78:B78"/>
@@ -7967,28 +7972,28 @@
       </c>
     </row>
     <row r="6" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="75" t="s">
+      <c r="A6" s="80" t="s">
         <v>272</v>
       </c>
-      <c r="B6" s="75"/>
+      <c r="B6" s="80"/>
       <c r="E6" s="42" t="s">
         <v>277</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="39" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="75" t="s">
+      <c r="A7" s="80" t="s">
         <v>273</v>
       </c>
-      <c r="B7" s="75"/>
+      <c r="B7" s="80"/>
       <c r="E7" s="42" t="s">
         <v>278</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="47" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="75" t="s">
+      <c r="A8" s="80" t="s">
         <v>274</v>
       </c>
-      <c r="B8" s="75"/>
+      <c r="B8" s="80"/>
       <c r="E8" s="42" t="s">
         <v>279</v>
       </c>
@@ -8003,10 +8008,10 @@
       </c>
     </row>
     <row r="10" spans="1:8" ht="34" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="75" t="s">
+      <c r="A10" s="80" t="s">
         <v>276</v>
       </c>
-      <c r="B10" s="75"/>
+      <c r="B10" s="80"/>
       <c r="E10" s="40" t="s">
         <v>281</v>
       </c>
@@ -8580,10 +8585,10 @@
       <c r="H62" s="32"/>
     </row>
     <row r="63" spans="1:8" ht="22" x14ac:dyDescent="0.2">
-      <c r="A63" s="77" t="s">
+      <c r="A63" s="90" t="s">
         <v>481</v>
       </c>
-      <c r="B63" s="77"/>
+      <c r="B63" s="90"/>
     </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
@@ -8656,18 +8661,19 @@
       <c r="E93" s="10"/>
     </row>
   </sheetData>
+  <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="11">
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="A63:B63"/>
     <mergeCell ref="A72:B72"/>
     <mergeCell ref="A69:B69"/>
     <mergeCell ref="A66:B66"/>
     <mergeCell ref="A67:B67"/>
     <mergeCell ref="A70:B70"/>
     <mergeCell ref="A71:B71"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="A63:B63"/>
   </mergeCells>
   <conditionalFormatting sqref="F54:F59">
     <cfRule type="containsText" dxfId="7" priority="2" operator="containsText" text="additional">
@@ -8743,12 +8749,12 @@
       </c>
     </row>
     <row r="6" spans="1:13" ht="39" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="75" t="s">
+      <c r="A6" s="80" t="s">
         <v>314</v>
       </c>
-      <c r="B6" s="75"/>
-      <c r="C6" s="75"/>
-      <c r="D6" s="75"/>
+      <c r="B6" s="80"/>
+      <c r="C6" s="80"/>
+      <c r="D6" s="80"/>
       <c r="E6" s="23"/>
       <c r="G6" s="34" t="s">
         <v>318</v>
@@ -8756,12 +8762,12 @@
       <c r="H6" s="16"/>
     </row>
     <row r="7" spans="1:13" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="75" t="s">
+      <c r="A7" s="80" t="s">
         <v>317</v>
       </c>
-      <c r="B7" s="75"/>
-      <c r="C7" s="75"/>
-      <c r="D7" s="75"/>
+      <c r="B7" s="80"/>
+      <c r="C7" s="80"/>
+      <c r="D7" s="80"/>
       <c r="E7" s="23"/>
       <c r="F7" s="23"/>
       <c r="G7" t="s">
@@ -8769,20 +8775,20 @@
       </c>
     </row>
     <row r="8" spans="1:13" ht="57" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="75" t="s">
+      <c r="A8" s="80" t="s">
         <v>316</v>
       </c>
-      <c r="B8" s="75"/>
-      <c r="C8" s="75"/>
-      <c r="D8" s="75"/>
+      <c r="B8" s="80"/>
+      <c r="C8" s="80"/>
+      <c r="D8" s="80"/>
       <c r="E8" s="23"/>
       <c r="F8" s="23"/>
-      <c r="G8" s="75" t="s">
+      <c r="G8" s="80" t="s">
         <v>320</v>
       </c>
-      <c r="H8" s="75"/>
-      <c r="I8" s="75"/>
-      <c r="J8" s="75"/>
+      <c r="H8" s="80"/>
+      <c r="I8" s="80"/>
+      <c r="J8" s="80"/>
       <c r="K8" s="23"/>
       <c r="L8" s="23"/>
       <c r="M8" s="23"/>
@@ -9344,10 +9350,10 @@
       <c r="M68" s="32"/>
     </row>
     <row r="70" spans="1:13" ht="22" x14ac:dyDescent="0.2">
-      <c r="A70" s="77" t="s">
+      <c r="A70" s="90" t="s">
         <v>372</v>
       </c>
-      <c r="B70" s="77"/>
+      <c r="B70" s="90"/>
     </row>
     <row r="71" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
@@ -9397,15 +9403,16 @@
       <c r="A105" s="3"/>
     </row>
   </sheetData>
+  <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="8">
+    <mergeCell ref="G8:J8"/>
+    <mergeCell ref="A70:B70"/>
     <mergeCell ref="A74:B74"/>
     <mergeCell ref="A75:B75"/>
     <mergeCell ref="A76:B76"/>
     <mergeCell ref="A6:D6"/>
     <mergeCell ref="A7:D7"/>
     <mergeCell ref="A8:D8"/>
-    <mergeCell ref="G8:J8"/>
-    <mergeCell ref="A70:B70"/>
   </mergeCells>
   <conditionalFormatting sqref="C31">
     <cfRule type="expression" dxfId="5" priority="1">
@@ -9475,22 +9482,22 @@
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A6" s="75" t="s">
+      <c r="A6" s="80" t="s">
         <v>376</v>
       </c>
-      <c r="B6" s="75"/>
-      <c r="C6" s="75"/>
-      <c r="D6" s="75"/>
-      <c r="E6" s="75"/>
+      <c r="B6" s="80"/>
+      <c r="C6" s="80"/>
+      <c r="D6" s="80"/>
+      <c r="E6" s="80"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A7" s="75" t="s">
+      <c r="A7" s="80" t="s">
         <v>377</v>
       </c>
-      <c r="B7" s="75"/>
-      <c r="C7" s="75"/>
-      <c r="D7" s="75"/>
-      <c r="E7" s="75"/>
+      <c r="B7" s="80"/>
+      <c r="C7" s="80"/>
+      <c r="D7" s="80"/>
+      <c r="E7" s="80"/>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" s="40" t="s">
@@ -9502,22 +9509,22 @@
       <c r="E8" s="40"/>
     </row>
     <row r="9" spans="1:10" ht="35" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="75" t="s">
+      <c r="A9" s="80" t="s">
         <v>379</v>
       </c>
-      <c r="B9" s="75"/>
-      <c r="C9" s="75"/>
-      <c r="D9" s="75"/>
-      <c r="E9" s="75"/>
+      <c r="B9" s="80"/>
+      <c r="C9" s="80"/>
+      <c r="D9" s="80"/>
+      <c r="E9" s="80"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A10" s="75" t="s">
+      <c r="A10" s="80" t="s">
         <v>380</v>
       </c>
-      <c r="B10" s="75"/>
-      <c r="C10" s="75"/>
-      <c r="D10" s="75"/>
-      <c r="E10" s="75"/>
+      <c r="B10" s="80"/>
+      <c r="C10" s="80"/>
+      <c r="D10" s="80"/>
+      <c r="E10" s="80"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" s="40" t="s">
@@ -9529,13 +9536,13 @@
       <c r="E11" s="40"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A12" s="75" t="s">
+      <c r="A12" s="80" t="s">
         <v>382</v>
       </c>
-      <c r="B12" s="75"/>
-      <c r="C12" s="75"/>
-      <c r="D12" s="75"/>
-      <c r="E12" s="75"/>
+      <c r="B12" s="80"/>
+      <c r="C12" s="80"/>
+      <c r="D12" s="80"/>
+      <c r="E12" s="80"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
@@ -10312,10 +10319,10 @@
       <c r="J114" s="32"/>
     </row>
     <row r="115" spans="1:14" ht="24" x14ac:dyDescent="0.2">
-      <c r="A115" s="83" t="s">
+      <c r="A115" s="87" t="s">
         <v>73</v>
       </c>
-      <c r="B115" s="83"/>
+      <c r="B115" s="87"/>
       <c r="N115" s="10"/>
     </row>
     <row r="116" spans="1:14" ht="19" x14ac:dyDescent="0.25">
@@ -10358,10 +10365,10 @@
       <c r="B121" s="78"/>
     </row>
     <row r="123" spans="1:14" ht="24" x14ac:dyDescent="0.2">
-      <c r="A123" s="83" t="s">
+      <c r="A123" s="87" t="s">
         <v>374</v>
       </c>
-      <c r="B123" s="83"/>
+      <c r="B123" s="87"/>
     </row>
     <row r="124" spans="1:14" ht="19" x14ac:dyDescent="0.25">
       <c r="A124" s="6" t="s">
@@ -10397,12 +10404,8 @@
       <c r="B131" s="78"/>
     </row>
   </sheetData>
+  <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="13">
-    <mergeCell ref="A12:E12"/>
-    <mergeCell ref="A6:E6"/>
-    <mergeCell ref="A7:E7"/>
-    <mergeCell ref="A9:E9"/>
-    <mergeCell ref="A10:E10"/>
     <mergeCell ref="A131:B131"/>
     <mergeCell ref="A119:B119"/>
     <mergeCell ref="A120:B120"/>
@@ -10411,6 +10414,11 @@
     <mergeCell ref="A123:B123"/>
     <mergeCell ref="A125:B125"/>
     <mergeCell ref="A128:B128"/>
+    <mergeCell ref="A12:E12"/>
+    <mergeCell ref="A6:E6"/>
+    <mergeCell ref="A7:E7"/>
+    <mergeCell ref="A9:E9"/>
+    <mergeCell ref="A10:E10"/>
   </mergeCells>
   <conditionalFormatting sqref="E11:E106">
     <cfRule type="containsText" dxfId="3" priority="3" operator="containsText" text="Medium">

</xml_diff>